<commit_message>
fix: some update in membrane protein
</commit_message>
<xml_diff>
--- a/data/sce_compartment_curation/Golgi_apparatus_annotations_v2.xlsx
+++ b/data/sce_compartment_curation/Golgi_apparatus_annotations_v2.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>YJL123C</t>
+          <t>YOR171C</t>
         </is>
       </c>
     </row>
@@ -451,7 +451,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>YKL034W</t>
+          <t>YER001W</t>
         </is>
       </c>
     </row>
@@ -461,7 +461,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>YNL029C</t>
+          <t>YIL014W</t>
         </is>
       </c>
     </row>
@@ -471,7 +471,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>YOR322C</t>
+          <t>YMR079W</t>
         </is>
       </c>
     </row>
@@ -481,7 +481,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>YGL210W</t>
+          <t>YJL204C</t>
         </is>
       </c>
     </row>
@@ -491,7 +491,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>YAR033W</t>
+          <t>YDR108W</t>
         </is>
       </c>
     </row>
@@ -501,7 +501,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>YLR242C</t>
+          <t>YOR070C</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>YPL246C</t>
+          <t>YOR036W</t>
         </is>
       </c>
     </row>
@@ -521,7 +521,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>YKL196C</t>
+          <t>YER005W</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>YJL029C</t>
+          <t>YNL044W</t>
         </is>
       </c>
     </row>
@@ -541,7 +541,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>YOL107W</t>
+          <t>YPL246C</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>YPL057C</t>
+          <t>YMR054W</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>YDR483W</t>
+          <t>YDR367W</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>YDR264C</t>
+          <t>YDL137W</t>
         </is>
       </c>
     </row>
@@ -581,7 +581,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>YJL186W</t>
+          <t>YBL069W</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>YMR292W</t>
+          <t>YDR372C</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>YHR123W</t>
+          <t>YNL130C</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>YCL057W</t>
+          <t>YNL029C</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>YDR351W</t>
+          <t>YKL196C</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>YLR309C</t>
+          <t>YDR137W</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>YMR079W</t>
+          <t>YGL257C</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>YDR108W</t>
+          <t>YJL186W</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>YJL139C</t>
+          <t>YEL042W</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>YLR220W</t>
+          <t>YER031C</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>YDL206W</t>
+          <t>YOR034C</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>YKL063C</t>
+          <t>YPL051W</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>YKL209C</t>
+          <t>YKL004W</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>YDR367W</t>
+          <t>YKL034W</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>YDR484W</t>
+          <t>YOR216C</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>YOR036W</t>
+          <t>YKR061W</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>YEL042W</t>
+          <t>YJL029C</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>YBR080C</t>
+          <t>YJR040W</t>
         </is>
       </c>
     </row>
@@ -771,7 +771,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>YDR372C</t>
+          <t>YKL063C</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>YNL024C-A</t>
+          <t>YBR015C</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>YER125W</t>
+          <t>YLR039C</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>YKL077W</t>
+          <t>YJR134C</t>
         </is>
       </c>
     </row>
@@ -811,7 +811,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>YER031C</t>
+          <t>YEL048C</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>YBR014C</t>
+          <t>YMR292W</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>YER001W</t>
+          <t>YDR351W</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>YPR113W</t>
+          <t>YER113C</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>YBR015C</t>
+          <t>YGL051W</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>YIL085C</t>
+          <t>YLR268W</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>YDR027C</t>
+          <t>YDR233C</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>YDL192W</t>
+          <t>YBL017C</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>YJL094C</t>
+          <t>YBR164C</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>YKL201C</t>
+          <t>YER125W</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>YOR099W</t>
+          <t>YAR033W</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>YPR165W</t>
+          <t>YCL057W</t>
         </is>
       </c>
     </row>
@@ -931,7 +931,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>YER005W</t>
+          <t>YDR027C</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>YOR216C</t>
+          <t>YLR260W</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>YOR034C</t>
+          <t>YBR036C</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>YMR054W</t>
+          <t>YDR264C</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>YOR171C</t>
+          <t>YLR242C</t>
         </is>
       </c>
     </row>
@@ -981,7 +981,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>YKL004W</t>
+          <t>YLR309C</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>YBL017C</t>
+          <t>YJL094C</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>YLR039C</t>
+          <t>YIL048W</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>YPL051W</t>
+          <t>YBR080C</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>YNL044W</t>
+          <t>YPL057C</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>YCR043C</t>
+          <t>YPR113W</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>YGL257C</t>
+          <t>YKL077W</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>YER113C</t>
+          <t>YGL210W</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>YDR137W</t>
+          <t>YDL206W</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>YBR161W</t>
+          <t>YOR322C</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>YBR164C</t>
+          <t>YBR014C</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>YLR268W</t>
+          <t>YOL107W</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>YOR070C</t>
+          <t>YLR220W</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>YBR199W</t>
+          <t>YDR484W</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>YDR233C</t>
+          <t>YDL010W</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>YLR262C</t>
+          <t>YPR165W</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>YNL183C</t>
+          <t>YPL204W</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>YJR134C</t>
+          <t>YOR099W</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>YNR026C</t>
+          <t>YJL139C</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>YBR036C</t>
+          <t>YIL085C</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>YKL174C</t>
+          <t>YNL183C</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>YKR020W</t>
+          <t>YKL201C</t>
         </is>
       </c>
     </row>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>YIL048W</t>
+          <t>YCR043C</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>YNL130C</t>
+          <t>YKL209C</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>YDL137W</t>
+          <t>YNL024C-A</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>YLR260W</t>
+          <t>YDL192W</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>YGL225W</t>
+          <t>YKR020W</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>YJR040W</t>
+          <t>YKL174C</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>YGL051W</t>
+          <t>YNR026C</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>YKR061W</t>
+          <t>YBR199W</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>YDL010W</t>
+          <t>YGL225W</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>YJL204C</t>
+          <t>YJL123C</t>
         </is>
       </c>
     </row>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>YBL069W</t>
+          <t>YLR262C</t>
         </is>
       </c>
     </row>
@@ -1321,7 +1321,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>YEL048C</t>
+          <t>YDR483W</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>YIL014W</t>
+          <t>YBR161W</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>YPL204W</t>
+          <t>YHR123W</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: update gene list belong to cell wall
</commit_message>
<xml_diff>
--- a/data/sce_compartment_curation/Golgi_apparatus_annotations_v2.xlsx
+++ b/data/sce_compartment_curation/Golgi_apparatus_annotations_v2.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>YKR061W</t>
+          <t>YOR216C</t>
         </is>
       </c>
     </row>
@@ -451,7 +451,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>YGL257C</t>
+          <t>YDR264C</t>
         </is>
       </c>
     </row>
@@ -461,7 +461,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>YER005W</t>
+          <t>YDR233C</t>
         </is>
       </c>
     </row>
@@ -471,7 +471,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>YPR165W</t>
+          <t>YJR134C</t>
         </is>
       </c>
     </row>
@@ -481,7 +481,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>YBR080C</t>
+          <t>YGL198W</t>
         </is>
       </c>
     </row>
@@ -491,7 +491,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>YER001W</t>
+          <t>YGL051W</t>
         </is>
       </c>
     </row>
@@ -501,7 +501,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>YKL174C</t>
+          <t>YLR262C</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>YPR113W</t>
+          <t>YDL206W</t>
         </is>
       </c>
     </row>
@@ -521,7 +521,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>YDR483W</t>
+          <t>YLR220W</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>YNL130C</t>
+          <t>YDR372C</t>
         </is>
       </c>
     </row>
@@ -541,7 +541,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>YKR020W</t>
+          <t>YJL139C</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>YEL042W</t>
+          <t>YOR070C</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>YDL010W</t>
+          <t>YPL057C</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>YER031C</t>
+          <t>YDL192W</t>
         </is>
       </c>
     </row>
@@ -581,7 +581,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>YNL029C</t>
+          <t>YBR164C</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>YHR123W</t>
+          <t>YBR036C</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>YGL198W</t>
+          <t>YKL063C</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>YLR039C</t>
+          <t>YBR199W</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>YCL057W</t>
+          <t>YLR268W</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>YGL210W</t>
+          <t>YPL246C</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>YJR134C</t>
+          <t>YLR260W</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>YOR171C</t>
+          <t>YMR054W</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>YJL094C</t>
+          <t>YOL107W</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>YBR161W</t>
+          <t>YEL048C</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>YKL004W</t>
+          <t>YOR322C</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>YDR372C</t>
+          <t>YDR484W</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>YER113C</t>
+          <t>YJL186W</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>YDR233C</t>
+          <t>YJL204C</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>YCR043C</t>
+          <t>YPR113W</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>YJL123C</t>
+          <t>YGL161C</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>YER125W</t>
+          <t>YER005W</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>YIL085C</t>
+          <t>YGL225W</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>YPL051W</t>
+          <t>YOR099W</t>
         </is>
       </c>
     </row>
@@ -771,7 +771,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>YBL017C</t>
+          <t>YER113C</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>YJL029C</t>
+          <t>YKL196C</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>YJR040W</t>
+          <t>YDR108W</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>YKL077W</t>
+          <t>YMR292W</t>
         </is>
       </c>
     </row>
@@ -811,7 +811,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>YNR026C</t>
+          <t>YKL034W</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>YMR292W</t>
+          <t>YNR026C</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>YOL107W</t>
+          <t>YGL257C</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>YMR054W</t>
+          <t>YJL094C</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>YPL204W</t>
+          <t>YDL137W</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>YDL192W</t>
+          <t>YKR061W</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>YKL209C</t>
+          <t>YDR351W</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>YNL024C-A</t>
+          <t>YAR033W</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>YDR027C</t>
+          <t>YJR040W</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>YDR351W</t>
+          <t>YOR171C</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>YLR220W</t>
+          <t>YKL077W</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>YLR262C</t>
+          <t>YDL010W</t>
         </is>
       </c>
     </row>
@@ -931,7 +931,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>YDR367W</t>
+          <t>YEL042W</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>YKL196C</t>
+          <t>YJL123C</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>YLR268W</t>
+          <t>YNL044W</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>YOR034C</t>
+          <t>YNL029C</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>YBR036C</t>
+          <t>YBL017C</t>
         </is>
       </c>
     </row>
@@ -981,7 +981,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>YGL161C</t>
+          <t>YDR137W</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>YJL204C</t>
+          <t>YPL204W</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>YOR099W</t>
+          <t>YBR161W</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>YPL057C</t>
+          <t>YDR483W</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>YOR216C</t>
+          <t>YLR242C</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>YLR242C</t>
+          <t>YPR165W</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>YDL137W</t>
+          <t>YKL209C</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>YBR164C</t>
+          <t>YBR015C</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>YMR079W</t>
+          <t>YNL024C-A</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>YLR260W</t>
+          <t>YIL014W</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>YGL225W</t>
+          <t>YIL048W</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>YBR014C</t>
+          <t>YPL051W</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>YDR264C</t>
+          <t>YKL004W</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>YOR322C</t>
+          <t>YHR123W</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>YKL063C</t>
+          <t>YJL029C</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>YJL139C</t>
+          <t>YOR036W</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>YIL014W</t>
+          <t>YKL201C</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>YOR036W</t>
+          <t>YDR027C</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>YOR070C</t>
+          <t>YNL130C</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>YDR484W</t>
+          <t>YOR034C</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>YLR309C</t>
+          <t>YGL210W</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>YIL048W</t>
+          <t>YDR367W</t>
         </is>
       </c>
     </row>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>YPL246C</t>
+          <t>YER125W</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>YDL206W</t>
+          <t>YCR043C</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>YDR137W</t>
+          <t>YKR020W</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>YNL183C</t>
+          <t>YLR039C</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>YAR033W</t>
+          <t>YKL174C</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>YBR015C</t>
+          <t>YBR080C</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>YDR108W</t>
+          <t>YBR014C</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>YKL201C</t>
+          <t>YER031C</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>YJL186W</t>
+          <t>YIL085C</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>YGL051W</t>
+          <t>YCL057W</t>
         </is>
       </c>
     </row>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>YEL048C</t>
+          <t>YER001W</t>
         </is>
       </c>
     </row>
@@ -1321,7 +1321,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>YBR199W</t>
+          <t>YLR309C</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>YKL034W</t>
+          <t>YMR079W</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>YNL044W</t>
+          <t>YNL183C</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: update some minor code
</commit_message>
<xml_diff>
--- a/data/sce_compartment_curation/Golgi_apparatus_annotations_v2.xlsx
+++ b/data/sce_compartment_curation/Golgi_apparatus_annotations_v2.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>YOR216C</t>
+          <t>YCR043C</t>
         </is>
       </c>
     </row>
@@ -451,7 +451,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>YDR264C</t>
+          <t>YOR322C</t>
         </is>
       </c>
     </row>
@@ -461,7 +461,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>YDR233C</t>
+          <t>YOR216C</t>
         </is>
       </c>
     </row>
@@ -471,7 +471,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>YJR134C</t>
+          <t>YOR036W</t>
         </is>
       </c>
     </row>
@@ -481,7 +481,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>YGL198W</t>
+          <t>YBR080C</t>
         </is>
       </c>
     </row>
@@ -491,7 +491,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>YGL051W</t>
+          <t>YCL057W</t>
         </is>
       </c>
     </row>
@@ -501,7 +501,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>YLR262C</t>
+          <t>YPR165W</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>YDL206W</t>
+          <t>YKL077W</t>
         </is>
       </c>
     </row>
@@ -521,7 +521,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>YLR220W</t>
+          <t>YNL183C</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>YDR372C</t>
+          <t>YPL204W</t>
         </is>
       </c>
     </row>
@@ -541,7 +541,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>YJL139C</t>
+          <t>YKL034W</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>YOR070C</t>
+          <t>YER113C</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>YPL057C</t>
+          <t>YBL069W</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>YDL192W</t>
+          <t>YJL094C</t>
         </is>
       </c>
     </row>
@@ -581,7 +581,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>YBR164C</t>
+          <t>YDR233C</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>YBR036C</t>
+          <t>YAR033W</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>YKL063C</t>
+          <t>YOR034C</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>YBR199W</t>
+          <t>YDR351W</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>YLR268W</t>
+          <t>YIL048W</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>YPL246C</t>
+          <t>YJL029C</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>YLR260W</t>
+          <t>YGL225W</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>YMR054W</t>
+          <t>YPL246C</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>YOL107W</t>
+          <t>YMR079W</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>YEL048C</t>
+          <t>YGL210W</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>YOR322C</t>
+          <t>YJR134C</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>YDR484W</t>
+          <t>YBR036C</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>YJL186W</t>
+          <t>YDR137W</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>YJL204C</t>
+          <t>YKL209C</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>YPR113W</t>
+          <t>YBL017C</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>YGL161C</t>
+          <t>YPL057C</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>YER005W</t>
+          <t>YLR039C</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>YGL225W</t>
+          <t>YLR220W</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>YOR099W</t>
+          <t>YDL137W</t>
         </is>
       </c>
     </row>
@@ -771,7 +771,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>YER113C</t>
+          <t>YJR040W</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>YKL196C</t>
+          <t>YDR367W</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>YDR108W</t>
+          <t>YPL051W</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>YMR292W</t>
+          <t>YOR171C</t>
         </is>
       </c>
     </row>
@@ -811,7 +811,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>YKL034W</t>
+          <t>YLR260W</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>YNR026C</t>
+          <t>YJL204C</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>YGL257C</t>
+          <t>YPR113W</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>YJL094C</t>
+          <t>YEL042W</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>YDL137W</t>
+          <t>YGL198W</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>YKR061W</t>
+          <t>YLR268W</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>YDR351W</t>
+          <t>YDL206W</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>YAR033W</t>
+          <t>YIL085C</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>YJR040W</t>
+          <t>YKL196C</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>YOR171C</t>
+          <t>YNR026C</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>YKL077W</t>
+          <t>YOR070C</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>YDL010W</t>
+          <t>YDR027C</t>
         </is>
       </c>
     </row>
@@ -931,7 +931,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>YEL042W</t>
+          <t>YDR264C</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>YJL123C</t>
+          <t>YNL130C</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>YNL044W</t>
+          <t>YEL048C</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>YNL029C</t>
+          <t>YGL161C</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>YBL017C</t>
+          <t>YOL107W</t>
         </is>
       </c>
     </row>
@@ -981,7 +981,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>YDR137W</t>
+          <t>YOR099W</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>YPL204W</t>
+          <t>YDL010W</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>YBR161W</t>
+          <t>YDR108W</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>YDR483W</t>
+          <t>YER125W</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>YLR242C</t>
+          <t>YBR015C</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>YPR165W</t>
+          <t>YMR054W</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>YKL209C</t>
+          <t>YKR061W</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>YBR015C</t>
+          <t>YJL139C</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>YNL024C-A</t>
+          <t>YBR014C</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>YIL014W</t>
+          <t>YHR123W</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>YIL048W</t>
+          <t>YLR262C</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>YPL051W</t>
+          <t>YKL174C</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>YKL004W</t>
+          <t>YDR483W</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>YHR123W</t>
+          <t>YBR199W</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>YJL029C</t>
+          <t>YKL201C</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>YOR036W</t>
+          <t>YNL044W</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>YKL201C</t>
+          <t>YER031C</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>YDR027C</t>
+          <t>YBR161W</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>YNL130C</t>
+          <t>YKR020W</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>YOR034C</t>
+          <t>YNL024C-A</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>YGL210W</t>
+          <t>YDR372C</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>YBL069W</t>
+          <t>YMR292W</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>YDR367W</t>
+          <t>YDL192W</t>
         </is>
       </c>
     </row>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>YER125W</t>
+          <t>YNL029C</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>YCR043C</t>
+          <t>YKL004W</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>YKR020W</t>
+          <t>YIL014W</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>YLR039C</t>
+          <t>YDR484W</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>YKL174C</t>
+          <t>YGL051W</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>YBR080C</t>
+          <t>YKL063C</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>YBR014C</t>
+          <t>YER005W</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>YER031C</t>
+          <t>YER001W</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>YIL085C</t>
+          <t>YGL257C</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>YCL057W</t>
+          <t>YJL123C</t>
         </is>
       </c>
     </row>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>YER001W</t>
+          <t>YLR309C</t>
         </is>
       </c>
     </row>
@@ -1321,7 +1321,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>YLR309C</t>
+          <t>YJL186W</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>YMR079W</t>
+          <t>YBR164C</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>YNL183C</t>
+          <t>YLR242C</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: update some results
</commit_message>
<xml_diff>
--- a/data/sce_compartment_curation/Golgi_apparatus_annotations_v2.xlsx
+++ b/data/sce_compartment_curation/Golgi_apparatus_annotations_v2.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>YNL029C</t>
+          <t>YER031C</t>
         </is>
       </c>
     </row>
@@ -451,7 +451,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>YLR309C</t>
+          <t>YJL094C</t>
         </is>
       </c>
     </row>
@@ -461,7 +461,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>YBR199W</t>
+          <t>YJL123C</t>
         </is>
       </c>
     </row>
@@ -471,7 +471,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>YJR134C</t>
+          <t>YKL004W</t>
         </is>
       </c>
     </row>
@@ -481,7 +481,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>YKL196C</t>
+          <t>YBR161W</t>
         </is>
       </c>
     </row>
@@ -491,7 +491,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>YJR040W</t>
+          <t>YLR262C</t>
         </is>
       </c>
     </row>
@@ -501,7 +501,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>YBR080C</t>
+          <t>YJR134C</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>YBR036C</t>
+          <t>YDR137W</t>
         </is>
       </c>
     </row>
@@ -521,7 +521,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>YJL204C</t>
+          <t>YDR264C</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>YHR123W</t>
+          <t>YCL057W</t>
         </is>
       </c>
     </row>
@@ -541,7 +541,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>YJL139C</t>
+          <t>YOR099W</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>YKL174C</t>
+          <t>YKL077W</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>YMR054W</t>
+          <t>YBR015C</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>YOR070C</t>
+          <t>YDL010W</t>
         </is>
       </c>
     </row>
@@ -581,7 +581,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>YDR233C</t>
+          <t>YJL139C</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>YER031C</t>
+          <t>YGL051W</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>YDR483W</t>
+          <t>YPL051W</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>YOR034C</t>
+          <t>YNL024C-A</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>YOL107W</t>
+          <t>YDR351W</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>YBR015C</t>
+          <t>YCR043C</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>YGL225W</t>
+          <t>YDR483W</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>YPR113W</t>
+          <t>YEL042W</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>YBR164C</t>
+          <t>YAR033W</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>YKL063C</t>
+          <t>YDR233C</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>YKL209C</t>
+          <t>YGL257C</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>YDR372C</t>
+          <t>YKL196C</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>YOR322C</t>
+          <t>YKR020W</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>YDR108W</t>
+          <t>YDL192W</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>YBR014C</t>
+          <t>YPL246C</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>YER113C</t>
+          <t>YLR220W</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>YDR027C</t>
+          <t>YJL186W</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>YLR242C</t>
+          <t>YMR292W</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>YGL210W</t>
+          <t>YNL130C</t>
         </is>
       </c>
     </row>
@@ -771,7 +771,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>YKL201C</t>
+          <t>YNL183C</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>YKR020W</t>
+          <t>YBR014C</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>YDR484W</t>
+          <t>YER113C</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>YEL042W</t>
+          <t>YER005W</t>
         </is>
       </c>
     </row>
@@ -811,7 +811,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>YKL034W</t>
+          <t>YOR070C</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>YLR268W</t>
+          <t>YIL085C</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>YMR292W</t>
+          <t>YJR040W</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>YOR171C</t>
+          <t>YDL206W</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>YDR137W</t>
+          <t>YNR026C</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>YOR036W</t>
+          <t>YDR367W</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>YNL183C</t>
+          <t>YER001W</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>YDL206W</t>
+          <t>YGL210W</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>YBL017C</t>
+          <t>YEL048C</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>YBL069W</t>
+          <t>YLR039C</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>YPL051W</t>
+          <t>YBL069W</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>YER005W</t>
+          <t>YBL017C</t>
         </is>
       </c>
     </row>
@@ -931,7 +931,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>YNL024C-A</t>
+          <t>YBR164C</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>YPL204W</t>
+          <t>YIL014W</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>YDR351W</t>
+          <t>YNL029C</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>YGL257C</t>
+          <t>YJL029C</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>YCR043C</t>
+          <t>YBR080C</t>
         </is>
       </c>
     </row>
@@ -981,7 +981,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>YJL123C</t>
+          <t>YGL161C</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>YLR039C</t>
+          <t>YKL034W</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>YER125W</t>
+          <t>YDR108W</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>YIL014W</t>
+          <t>YKL063C</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>YBR161W</t>
+          <t>YDR372C</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>YPL057C</t>
+          <t>YLR242C</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>YNL130C</t>
+          <t>YBR199W</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>YPR165W</t>
+          <t>YER125W</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>YJL186W</t>
+          <t>YKR061W</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>YKL077W</t>
+          <t>YKL209C</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>YOR216C</t>
+          <t>YOR034C</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>YDR264C</t>
+          <t>YBR036C</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>YGL051W</t>
+          <t>YOL107W</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>YJL029C</t>
+          <t>YPL204W</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>YNR026C</t>
+          <t>YMR054W</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>YDL137W</t>
+          <t>YKL201C</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>YAR033W</t>
+          <t>YHR123W</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>YLR260W</t>
+          <t>YPL057C</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>YLR220W</t>
+          <t>YOR322C</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>YOR099W</t>
+          <t>YDR027C</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>YNL044W</t>
+          <t>YPR165W</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>YEL048C</t>
+          <t>YOR216C</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>YDL192W</t>
+          <t>YOR171C</t>
         </is>
       </c>
     </row>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>YKR061W</t>
+          <t>YDR484W</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>YPL246C</t>
+          <t>YPR113W</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>YMR079W</t>
+          <t>YLR268W</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>YJL094C</t>
+          <t>YNL044W</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>YCL057W</t>
+          <t>YJL204C</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>YDL010W</t>
+          <t>YDL137W</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>YKL004W</t>
+          <t>YMR079W</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>YIL085C</t>
+          <t>YGL198W</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>YDR367W</t>
+          <t>YGL225W</t>
         </is>
       </c>
     </row>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>YLR262C</t>
+          <t>YOR036W</t>
         </is>
       </c>
     </row>
@@ -1321,7 +1321,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>YER001W</t>
+          <t>YLR260W</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>YGL198W</t>
+          <t>YLR309C</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>YGL161C</t>
+          <t>YKL174C</t>
         </is>
       </c>
     </row>

</xml_diff>